<commit_message>
Fix critico xlsx: MAXIFS necesita prefijo _xlfn. (daba #NAME? en Excel/LibreOffice)
- Cazado verificando el render real en LibreOffice (ya instalado): el PR flag
  mostraba #NAME? en cada celda. La lib formulas es indulgente y no lo detectaba.
- verify_tracker.py ahora recalcula con LibreOffice (autoritativo) + barrido de
  errores; cae a lib formulas si no esta instalado.
- Print setup (fit-to-width, landscape Dashboard, print areas) para impresion limpia.
- Ancho col PR ajustado. Mockups de listing reales (build_mockups.py) + entrega Google Sheets.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/products/Fitness_Tracker/Adaptive_Fitness_Tracker.xlsx
+++ b/products/Fitness_Tracker/Adaptive_Fitness_Tracker.xlsx
@@ -13,7 +13,13 @@
     <sheet name="Workout Log" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Guide" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Dashboard'!$A$1:$N$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Setup'!$A$1:$F$26</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Weight Log'!$3:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Workout Log'!$3:$3</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Guide'!$A$1:$A$25</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -726,7 +732,7 @@
   <sheetPr>
     <tabColor rgb="002563EB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -891,7 +897,8 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A16:C18"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -902,7 +909,7 @@
   <sheetPr>
     <tabColor rgb="000000FF"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1284,7 +1291,8 @@
       <formula1>"1.6,1.8,2.0,2.2"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="1" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -1293,7 +1301,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3283,7 +3291,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -3291,7 +3300,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3302,7 +3311,7 @@
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -3378,7 +3387,7 @@
         <v/>
       </c>
       <c r="G4" s="30">
-        <f>IF($F4="","",IF($F4&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B4),"PR ★",""))</f>
+        <f>IF($F4="","",IF($F4&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B4),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I4" s="14" t="inlineStr">
@@ -3410,7 +3419,7 @@
         <v/>
       </c>
       <c r="G5" s="30">
-        <f>IF($F5="","",IF($F5&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B5),"PR ★",""))</f>
+        <f>IF($F5="","",IF($F5&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B5),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I5" s="14" t="inlineStr">
@@ -3442,7 +3451,7 @@
         <v/>
       </c>
       <c r="G6" s="30">
-        <f>IF($F6="","",IF($F6&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B6),"PR ★",""))</f>
+        <f>IF($F6="","",IF($F6&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B6),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I6" s="14" t="inlineStr">
@@ -3474,7 +3483,7 @@
         <v/>
       </c>
       <c r="G7" s="30">
-        <f>IF($F7="","",IF($F7&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B7),"PR ★",""))</f>
+        <f>IF($F7="","",IF($F7&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B7),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I7" s="14" t="inlineStr">
@@ -3506,7 +3515,7 @@
         <v/>
       </c>
       <c r="G8" s="30">
-        <f>IF($F8="","",IF($F8&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B8),"PR ★",""))</f>
+        <f>IF($F8="","",IF($F8&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B8),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I8" s="14" t="inlineStr">
@@ -3538,7 +3547,7 @@
         <v/>
       </c>
       <c r="G9" s="30">
-        <f>IF($F9="","",IF($F9&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B9),"PR ★",""))</f>
+        <f>IF($F9="","",IF($F9&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B9),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I9" s="14" t="inlineStr">
@@ -3555,7 +3564,7 @@
         <v/>
       </c>
       <c r="G10" s="30">
-        <f>IF($F10="","",IF($F10&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B10),"PR ★",""))</f>
+        <f>IF($F10="","",IF($F10&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B10),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I10" s="14" t="inlineStr">
@@ -3572,7 +3581,7 @@
         <v/>
       </c>
       <c r="G11" s="30">
-        <f>IF($F11="","",IF($F11&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B11),"PR ★",""))</f>
+        <f>IF($F11="","",IF($F11&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B11),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I11" s="14" t="inlineStr">
@@ -3589,7 +3598,7 @@
         <v/>
       </c>
       <c r="G12" s="30">
-        <f>IF($F12="","",IF($F12&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B12),"PR ★",""))</f>
+        <f>IF($F12="","",IF($F12&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B12),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I12" s="14" t="inlineStr">
@@ -3606,7 +3615,7 @@
         <v/>
       </c>
       <c r="G13" s="30">
-        <f>IF($F13="","",IF($F13&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B13),"PR ★",""))</f>
+        <f>IF($F13="","",IF($F13&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B13),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I13" s="14" t="inlineStr">
@@ -3623,7 +3632,7 @@
         <v/>
       </c>
       <c r="G14" s="30">
-        <f>IF($F14="","",IF($F14&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B14),"PR ★",""))</f>
+        <f>IF($F14="","",IF($F14&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B14),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I14" s="14" t="inlineStr">
@@ -3640,7 +3649,7 @@
         <v/>
       </c>
       <c r="G15" s="30">
-        <f>IF($F15="","",IF($F15&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B15),"PR ★",""))</f>
+        <f>IF($F15="","",IF($F15&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B15),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I15" s="14" t="inlineStr">
@@ -3657,7 +3666,7 @@
         <v/>
       </c>
       <c r="G16" s="30">
-        <f>IF($F16="","",IF($F16&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B16),"PR ★",""))</f>
+        <f>IF($F16="","",IF($F16&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B16),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I16" s="14" t="inlineStr">
@@ -3674,7 +3683,7 @@
         <v/>
       </c>
       <c r="G17" s="30">
-        <f>IF($F17="","",IF($F17&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B17),"PR ★",""))</f>
+        <f>IF($F17="","",IF($F17&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B17),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I17" s="14" t="inlineStr">
@@ -3691,7 +3700,7 @@
         <v/>
       </c>
       <c r="G18" s="30">
-        <f>IF($F18="","",IF($F18&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B18),"PR ★",""))</f>
+        <f>IF($F18="","",IF($F18&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B18),"PR ★",""))</f>
         <v/>
       </c>
       <c r="I18" s="14" t="inlineStr">
@@ -3708,7 +3717,7 @@
         <v/>
       </c>
       <c r="G19" s="30">
-        <f>IF($F19="","",IF($F19&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B19),"PR ★",""))</f>
+        <f>IF($F19="","",IF($F19&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B19),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3720,7 +3729,7 @@
         <v/>
       </c>
       <c r="G20" s="30">
-        <f>IF($F20="","",IF($F20&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B20),"PR ★",""))</f>
+        <f>IF($F20="","",IF($F20&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B20),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3732,7 +3741,7 @@
         <v/>
       </c>
       <c r="G21" s="30">
-        <f>IF($F21="","",IF($F21&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B21),"PR ★",""))</f>
+        <f>IF($F21="","",IF($F21&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B21),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3744,7 +3753,7 @@
         <v/>
       </c>
       <c r="G22" s="30">
-        <f>IF($F22="","",IF($F22&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B22),"PR ★",""))</f>
+        <f>IF($F22="","",IF($F22&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B22),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3756,7 +3765,7 @@
         <v/>
       </c>
       <c r="G23" s="30">
-        <f>IF($F23="","",IF($F23&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B23),"PR ★",""))</f>
+        <f>IF($F23="","",IF($F23&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B23),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3768,7 +3777,7 @@
         <v/>
       </c>
       <c r="G24" s="30">
-        <f>IF($F24="","",IF($F24&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B24),"PR ★",""))</f>
+        <f>IF($F24="","",IF($F24&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B24),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3780,7 +3789,7 @@
         <v/>
       </c>
       <c r="G25" s="30">
-        <f>IF($F25="","",IF($F25&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B25),"PR ★",""))</f>
+        <f>IF($F25="","",IF($F25&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B25),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3792,7 +3801,7 @@
         <v/>
       </c>
       <c r="G26" s="30">
-        <f>IF($F26="","",IF($F26&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B26),"PR ★",""))</f>
+        <f>IF($F26="","",IF($F26&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B26),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3804,7 +3813,7 @@
         <v/>
       </c>
       <c r="G27" s="30">
-        <f>IF($F27="","",IF($F27&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B27),"PR ★",""))</f>
+        <f>IF($F27="","",IF($F27&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B27),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3816,7 +3825,7 @@
         <v/>
       </c>
       <c r="G28" s="30">
-        <f>IF($F28="","",IF($F28&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B28),"PR ★",""))</f>
+        <f>IF($F28="","",IF($F28&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B28),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3828,7 +3837,7 @@
         <v/>
       </c>
       <c r="G29" s="30">
-        <f>IF($F29="","",IF($F29&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B29),"PR ★",""))</f>
+        <f>IF($F29="","",IF($F29&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B29),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3840,7 +3849,7 @@
         <v/>
       </c>
       <c r="G30" s="30">
-        <f>IF($F30="","",IF($F30&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B30),"PR ★",""))</f>
+        <f>IF($F30="","",IF($F30&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B30),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3852,7 +3861,7 @@
         <v/>
       </c>
       <c r="G31" s="30">
-        <f>IF($F31="","",IF($F31&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B31),"PR ★",""))</f>
+        <f>IF($F31="","",IF($F31&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B31),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3864,7 +3873,7 @@
         <v/>
       </c>
       <c r="G32" s="30">
-        <f>IF($F32="","",IF($F32&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B32),"PR ★",""))</f>
+        <f>IF($F32="","",IF($F32&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B32),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3876,7 +3885,7 @@
         <v/>
       </c>
       <c r="G33" s="30">
-        <f>IF($F33="","",IF($F33&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B33),"PR ★",""))</f>
+        <f>IF($F33="","",IF($F33&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B33),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3888,7 +3897,7 @@
         <v/>
       </c>
       <c r="G34" s="30">
-        <f>IF($F34="","",IF($F34&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B34),"PR ★",""))</f>
+        <f>IF($F34="","",IF($F34&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B34),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3900,7 +3909,7 @@
         <v/>
       </c>
       <c r="G35" s="30">
-        <f>IF($F35="","",IF($F35&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B35),"PR ★",""))</f>
+        <f>IF($F35="","",IF($F35&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B35),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3912,7 +3921,7 @@
         <v/>
       </c>
       <c r="G36" s="30">
-        <f>IF($F36="","",IF($F36&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B36),"PR ★",""))</f>
+        <f>IF($F36="","",IF($F36&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B36),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3924,7 +3933,7 @@
         <v/>
       </c>
       <c r="G37" s="30">
-        <f>IF($F37="","",IF($F37&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B37),"PR ★",""))</f>
+        <f>IF($F37="","",IF($F37&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B37),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3936,7 +3945,7 @@
         <v/>
       </c>
       <c r="G38" s="30">
-        <f>IF($F38="","",IF($F38&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B38),"PR ★",""))</f>
+        <f>IF($F38="","",IF($F38&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B38),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3948,7 +3957,7 @@
         <v/>
       </c>
       <c r="G39" s="30">
-        <f>IF($F39="","",IF($F39&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B39),"PR ★",""))</f>
+        <f>IF($F39="","",IF($F39&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B39),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3960,7 +3969,7 @@
         <v/>
       </c>
       <c r="G40" s="30">
-        <f>IF($F40="","",IF($F40&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B40),"PR ★",""))</f>
+        <f>IF($F40="","",IF($F40&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B40),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3972,7 +3981,7 @@
         <v/>
       </c>
       <c r="G41" s="30">
-        <f>IF($F41="","",IF($F41&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B41),"PR ★",""))</f>
+        <f>IF($F41="","",IF($F41&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B41),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3984,7 +3993,7 @@
         <v/>
       </c>
       <c r="G42" s="30">
-        <f>IF($F42="","",IF($F42&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B42),"PR ★",""))</f>
+        <f>IF($F42="","",IF($F42&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B42),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -3996,7 +4005,7 @@
         <v/>
       </c>
       <c r="G43" s="30">
-        <f>IF($F43="","",IF($F43&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B43),"PR ★",""))</f>
+        <f>IF($F43="","",IF($F43&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B43),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4008,7 +4017,7 @@
         <v/>
       </c>
       <c r="G44" s="30">
-        <f>IF($F44="","",IF($F44&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B44),"PR ★",""))</f>
+        <f>IF($F44="","",IF($F44&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B44),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4020,7 +4029,7 @@
         <v/>
       </c>
       <c r="G45" s="30">
-        <f>IF($F45="","",IF($F45&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B45),"PR ★",""))</f>
+        <f>IF($F45="","",IF($F45&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B45),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4032,7 +4041,7 @@
         <v/>
       </c>
       <c r="G46" s="30">
-        <f>IF($F46="","",IF($F46&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B46),"PR ★",""))</f>
+        <f>IF($F46="","",IF($F46&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B46),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4044,7 +4053,7 @@
         <v/>
       </c>
       <c r="G47" s="30">
-        <f>IF($F47="","",IF($F47&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B47),"PR ★",""))</f>
+        <f>IF($F47="","",IF($F47&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B47),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4056,7 +4065,7 @@
         <v/>
       </c>
       <c r="G48" s="30">
-        <f>IF($F48="","",IF($F48&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B48),"PR ★",""))</f>
+        <f>IF($F48="","",IF($F48&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B48),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4068,7 +4077,7 @@
         <v/>
       </c>
       <c r="G49" s="30">
-        <f>IF($F49="","",IF($F49&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B49),"PR ★",""))</f>
+        <f>IF($F49="","",IF($F49&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B49),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4080,7 +4089,7 @@
         <v/>
       </c>
       <c r="G50" s="30">
-        <f>IF($F50="","",IF($F50&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B50),"PR ★",""))</f>
+        <f>IF($F50="","",IF($F50&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B50),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4092,7 +4101,7 @@
         <v/>
       </c>
       <c r="G51" s="30">
-        <f>IF($F51="","",IF($F51&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B51),"PR ★",""))</f>
+        <f>IF($F51="","",IF($F51&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B51),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4104,7 +4113,7 @@
         <v/>
       </c>
       <c r="G52" s="30">
-        <f>IF($F52="","",IF($F52&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B52),"PR ★",""))</f>
+        <f>IF($F52="","",IF($F52&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B52),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4116,7 +4125,7 @@
         <v/>
       </c>
       <c r="G53" s="30">
-        <f>IF($F53="","",IF($F53&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B53),"PR ★",""))</f>
+        <f>IF($F53="","",IF($F53&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B53),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4128,7 +4137,7 @@
         <v/>
       </c>
       <c r="G54" s="30">
-        <f>IF($F54="","",IF($F54&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B54),"PR ★",""))</f>
+        <f>IF($F54="","",IF($F54&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B54),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4140,7 +4149,7 @@
         <v/>
       </c>
       <c r="G55" s="30">
-        <f>IF($F55="","",IF($F55&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B55),"PR ★",""))</f>
+        <f>IF($F55="","",IF($F55&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B55),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4152,7 +4161,7 @@
         <v/>
       </c>
       <c r="G56" s="30">
-        <f>IF($F56="","",IF($F56&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B56),"PR ★",""))</f>
+        <f>IF($F56="","",IF($F56&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B56),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4164,7 +4173,7 @@
         <v/>
       </c>
       <c r="G57" s="30">
-        <f>IF($F57="","",IF($F57&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B57),"PR ★",""))</f>
+        <f>IF($F57="","",IF($F57&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B57),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4176,7 +4185,7 @@
         <v/>
       </c>
       <c r="G58" s="30">
-        <f>IF($F58="","",IF($F58&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B58),"PR ★",""))</f>
+        <f>IF($F58="","",IF($F58&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B58),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4188,7 +4197,7 @@
         <v/>
       </c>
       <c r="G59" s="30">
-        <f>IF($F59="","",IF($F59&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B59),"PR ★",""))</f>
+        <f>IF($F59="","",IF($F59&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B59),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4200,7 +4209,7 @@
         <v/>
       </c>
       <c r="G60" s="30">
-        <f>IF($F60="","",IF($F60&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B60),"PR ★",""))</f>
+        <f>IF($F60="","",IF($F60&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B60),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4212,7 +4221,7 @@
         <v/>
       </c>
       <c r="G61" s="30">
-        <f>IF($F61="","",IF($F61&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B61),"PR ★",""))</f>
+        <f>IF($F61="","",IF($F61&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B61),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4224,7 +4233,7 @@
         <v/>
       </c>
       <c r="G62" s="30">
-        <f>IF($F62="","",IF($F62&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B62),"PR ★",""))</f>
+        <f>IF($F62="","",IF($F62&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B62),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4236,7 +4245,7 @@
         <v/>
       </c>
       <c r="G63" s="30">
-        <f>IF($F63="","",IF($F63&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B63),"PR ★",""))</f>
+        <f>IF($F63="","",IF($F63&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B63),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4248,7 +4257,7 @@
         <v/>
       </c>
       <c r="G64" s="30">
-        <f>IF($F64="","",IF($F64&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B64),"PR ★",""))</f>
+        <f>IF($F64="","",IF($F64&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B64),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4260,7 +4269,7 @@
         <v/>
       </c>
       <c r="G65" s="30">
-        <f>IF($F65="","",IF($F65&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B65),"PR ★",""))</f>
+        <f>IF($F65="","",IF($F65&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B65),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4272,7 +4281,7 @@
         <v/>
       </c>
       <c r="G66" s="30">
-        <f>IF($F66="","",IF($F66&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B66),"PR ★",""))</f>
+        <f>IF($F66="","",IF($F66&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B66),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4284,7 +4293,7 @@
         <v/>
       </c>
       <c r="G67" s="30">
-        <f>IF($F67="","",IF($F67&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B67),"PR ★",""))</f>
+        <f>IF($F67="","",IF($F67&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B67),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4296,7 +4305,7 @@
         <v/>
       </c>
       <c r="G68" s="30">
-        <f>IF($F68="","",IF($F68&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B68),"PR ★",""))</f>
+        <f>IF($F68="","",IF($F68&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B68),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4308,7 +4317,7 @@
         <v/>
       </c>
       <c r="G69" s="30">
-        <f>IF($F69="","",IF($F69&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B69),"PR ★",""))</f>
+        <f>IF($F69="","",IF($F69&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B69),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4320,7 +4329,7 @@
         <v/>
       </c>
       <c r="G70" s="30">
-        <f>IF($F70="","",IF($F70&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B70),"PR ★",""))</f>
+        <f>IF($F70="","",IF($F70&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B70),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4332,7 +4341,7 @@
         <v/>
       </c>
       <c r="G71" s="30">
-        <f>IF($F71="","",IF($F71&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B71),"PR ★",""))</f>
+        <f>IF($F71="","",IF($F71&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B71),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4344,7 +4353,7 @@
         <v/>
       </c>
       <c r="G72" s="30">
-        <f>IF($F72="","",IF($F72&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B72),"PR ★",""))</f>
+        <f>IF($F72="","",IF($F72&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B72),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4356,7 +4365,7 @@
         <v/>
       </c>
       <c r="G73" s="30">
-        <f>IF($F73="","",IF($F73&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B73),"PR ★",""))</f>
+        <f>IF($F73="","",IF($F73&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B73),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4368,7 +4377,7 @@
         <v/>
       </c>
       <c r="G74" s="30">
-        <f>IF($F74="","",IF($F74&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B74),"PR ★",""))</f>
+        <f>IF($F74="","",IF($F74&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B74),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4380,7 +4389,7 @@
         <v/>
       </c>
       <c r="G75" s="30">
-        <f>IF($F75="","",IF($F75&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B75),"PR ★",""))</f>
+        <f>IF($F75="","",IF($F75&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B75),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4392,7 +4401,7 @@
         <v/>
       </c>
       <c r="G76" s="30">
-        <f>IF($F76="","",IF($F76&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B76),"PR ★",""))</f>
+        <f>IF($F76="","",IF($F76&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B76),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4404,7 +4413,7 @@
         <v/>
       </c>
       <c r="G77" s="30">
-        <f>IF($F77="","",IF($F77&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B77),"PR ★",""))</f>
+        <f>IF($F77="","",IF($F77&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B77),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4416,7 +4425,7 @@
         <v/>
       </c>
       <c r="G78" s="30">
-        <f>IF($F78="","",IF($F78&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B78),"PR ★",""))</f>
+        <f>IF($F78="","",IF($F78&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B78),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4428,7 +4437,7 @@
         <v/>
       </c>
       <c r="G79" s="30">
-        <f>IF($F79="","",IF($F79&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B79),"PR ★",""))</f>
+        <f>IF($F79="","",IF($F79&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B79),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4440,7 +4449,7 @@
         <v/>
       </c>
       <c r="G80" s="30">
-        <f>IF($F80="","",IF($F80&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B80),"PR ★",""))</f>
+        <f>IF($F80="","",IF($F80&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B80),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4452,7 +4461,7 @@
         <v/>
       </c>
       <c r="G81" s="30">
-        <f>IF($F81="","",IF($F81&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B81),"PR ★",""))</f>
+        <f>IF($F81="","",IF($F81&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B81),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4464,7 +4473,7 @@
         <v/>
       </c>
       <c r="G82" s="30">
-        <f>IF($F82="","",IF($F82&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B82),"PR ★",""))</f>
+        <f>IF($F82="","",IF($F82&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B82),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4476,7 +4485,7 @@
         <v/>
       </c>
       <c r="G83" s="30">
-        <f>IF($F83="","",IF($F83&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B83),"PR ★",""))</f>
+        <f>IF($F83="","",IF($F83&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B83),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4488,7 +4497,7 @@
         <v/>
       </c>
       <c r="G84" s="30">
-        <f>IF($F84="","",IF($F84&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B84),"PR ★",""))</f>
+        <f>IF($F84="","",IF($F84&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B84),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4500,7 +4509,7 @@
         <v/>
       </c>
       <c r="G85" s="30">
-        <f>IF($F85="","",IF($F85&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B85),"PR ★",""))</f>
+        <f>IF($F85="","",IF($F85&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B85),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4512,7 +4521,7 @@
         <v/>
       </c>
       <c r="G86" s="30">
-        <f>IF($F86="","",IF($F86&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B86),"PR ★",""))</f>
+        <f>IF($F86="","",IF($F86&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B86),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4524,7 +4533,7 @@
         <v/>
       </c>
       <c r="G87" s="30">
-        <f>IF($F87="","",IF($F87&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B87),"PR ★",""))</f>
+        <f>IF($F87="","",IF($F87&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B87),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4536,7 +4545,7 @@
         <v/>
       </c>
       <c r="G88" s="30">
-        <f>IF($F88="","",IF($F88&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B88),"PR ★",""))</f>
+        <f>IF($F88="","",IF($F88&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B88),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4548,7 +4557,7 @@
         <v/>
       </c>
       <c r="G89" s="30">
-        <f>IF($F89="","",IF($F89&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B89),"PR ★",""))</f>
+        <f>IF($F89="","",IF($F89&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B89),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4560,7 +4569,7 @@
         <v/>
       </c>
       <c r="G90" s="30">
-        <f>IF($F90="","",IF($F90&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B90),"PR ★",""))</f>
+        <f>IF($F90="","",IF($F90&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B90),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4572,7 +4581,7 @@
         <v/>
       </c>
       <c r="G91" s="30">
-        <f>IF($F91="","",IF($F91&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B91),"PR ★",""))</f>
+        <f>IF($F91="","",IF($F91&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B91),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4584,7 +4593,7 @@
         <v/>
       </c>
       <c r="G92" s="30">
-        <f>IF($F92="","",IF($F92&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B92),"PR ★",""))</f>
+        <f>IF($F92="","",IF($F92&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B92),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4596,7 +4605,7 @@
         <v/>
       </c>
       <c r="G93" s="30">
-        <f>IF($F93="","",IF($F93&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B93),"PR ★",""))</f>
+        <f>IF($F93="","",IF($F93&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B93),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4608,7 +4617,7 @@
         <v/>
       </c>
       <c r="G94" s="30">
-        <f>IF($F94="","",IF($F94&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B94),"PR ★",""))</f>
+        <f>IF($F94="","",IF($F94&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B94),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4620,7 +4629,7 @@
         <v/>
       </c>
       <c r="G95" s="30">
-        <f>IF($F95="","",IF($F95&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B95),"PR ★",""))</f>
+        <f>IF($F95="","",IF($F95&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B95),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4632,7 +4641,7 @@
         <v/>
       </c>
       <c r="G96" s="30">
-        <f>IF($F96="","",IF($F96&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B96),"PR ★",""))</f>
+        <f>IF($F96="","",IF($F96&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B96),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4644,7 +4653,7 @@
         <v/>
       </c>
       <c r="G97" s="30">
-        <f>IF($F97="","",IF($F97&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B97),"PR ★",""))</f>
+        <f>IF($F97="","",IF($F97&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B97),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4656,7 +4665,7 @@
         <v/>
       </c>
       <c r="G98" s="30">
-        <f>IF($F98="","",IF($F98&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B98),"PR ★",""))</f>
+        <f>IF($F98="","",IF($F98&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B98),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4668,7 +4677,7 @@
         <v/>
       </c>
       <c r="G99" s="30">
-        <f>IF($F99="","",IF($F99&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B99),"PR ★",""))</f>
+        <f>IF($F99="","",IF($F99&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B99),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4680,7 +4689,7 @@
         <v/>
       </c>
       <c r="G100" s="30">
-        <f>IF($F100="","",IF($F100&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B100),"PR ★",""))</f>
+        <f>IF($F100="","",IF($F100&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B100),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4692,7 +4701,7 @@
         <v/>
       </c>
       <c r="G101" s="30">
-        <f>IF($F101="","",IF($F101&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B101),"PR ★",""))</f>
+        <f>IF($F101="","",IF($F101&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B101),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4704,7 +4713,7 @@
         <v/>
       </c>
       <c r="G102" s="30">
-        <f>IF($F102="","",IF($F102&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B102),"PR ★",""))</f>
+        <f>IF($F102="","",IF($F102&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B102),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4716,7 +4725,7 @@
         <v/>
       </c>
       <c r="G103" s="30">
-        <f>IF($F103="","",IF($F103&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B103),"PR ★",""))</f>
+        <f>IF($F103="","",IF($F103&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B103),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4728,7 +4737,7 @@
         <v/>
       </c>
       <c r="G104" s="30">
-        <f>IF($F104="","",IF($F104&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B104),"PR ★",""))</f>
+        <f>IF($F104="","",IF($F104&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B104),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4740,7 +4749,7 @@
         <v/>
       </c>
       <c r="G105" s="30">
-        <f>IF($F105="","",IF($F105&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B105),"PR ★",""))</f>
+        <f>IF($F105="","",IF($F105&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B105),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4752,7 +4761,7 @@
         <v/>
       </c>
       <c r="G106" s="30">
-        <f>IF($F106="","",IF($F106&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B106),"PR ★",""))</f>
+        <f>IF($F106="","",IF($F106&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B106),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4764,7 +4773,7 @@
         <v/>
       </c>
       <c r="G107" s="30">
-        <f>IF($F107="","",IF($F107&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B107),"PR ★",""))</f>
+        <f>IF($F107="","",IF($F107&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B107),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4776,7 +4785,7 @@
         <v/>
       </c>
       <c r="G108" s="30">
-        <f>IF($F108="","",IF($F108&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B108),"PR ★",""))</f>
+        <f>IF($F108="","",IF($F108&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B108),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4788,7 +4797,7 @@
         <v/>
       </c>
       <c r="G109" s="30">
-        <f>IF($F109="","",IF($F109&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B109),"PR ★",""))</f>
+        <f>IF($F109="","",IF($F109&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B109),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4800,7 +4809,7 @@
         <v/>
       </c>
       <c r="G110" s="30">
-        <f>IF($F110="","",IF($F110&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B110),"PR ★",""))</f>
+        <f>IF($F110="","",IF($F110&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B110),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4812,7 +4821,7 @@
         <v/>
       </c>
       <c r="G111" s="30">
-        <f>IF($F111="","",IF($F111&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B111),"PR ★",""))</f>
+        <f>IF($F111="","",IF($F111&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B111),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4824,7 +4833,7 @@
         <v/>
       </c>
       <c r="G112" s="30">
-        <f>IF($F112="","",IF($F112&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B112),"PR ★",""))</f>
+        <f>IF($F112="","",IF($F112&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B112),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4836,7 +4845,7 @@
         <v/>
       </c>
       <c r="G113" s="30">
-        <f>IF($F113="","",IF($F113&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B113),"PR ★",""))</f>
+        <f>IF($F113="","",IF($F113&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B113),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4848,7 +4857,7 @@
         <v/>
       </c>
       <c r="G114" s="30">
-        <f>IF($F114="","",IF($F114&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B114),"PR ★",""))</f>
+        <f>IF($F114="","",IF($F114&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B114),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4860,7 +4869,7 @@
         <v/>
       </c>
       <c r="G115" s="30">
-        <f>IF($F115="","",IF($F115&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B115),"PR ★",""))</f>
+        <f>IF($F115="","",IF($F115&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B115),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4872,7 +4881,7 @@
         <v/>
       </c>
       <c r="G116" s="30">
-        <f>IF($F116="","",IF($F116&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B116),"PR ★",""))</f>
+        <f>IF($F116="","",IF($F116&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B116),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4884,7 +4893,7 @@
         <v/>
       </c>
       <c r="G117" s="30">
-        <f>IF($F117="","",IF($F117&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B117),"PR ★",""))</f>
+        <f>IF($F117="","",IF($F117&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B117),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4896,7 +4905,7 @@
         <v/>
       </c>
       <c r="G118" s="30">
-        <f>IF($F118="","",IF($F118&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B118),"PR ★",""))</f>
+        <f>IF($F118="","",IF($F118&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B118),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4908,7 +4917,7 @@
         <v/>
       </c>
       <c r="G119" s="30">
-        <f>IF($F119="","",IF($F119&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B119),"PR ★",""))</f>
+        <f>IF($F119="","",IF($F119&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B119),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4920,7 +4929,7 @@
         <v/>
       </c>
       <c r="G120" s="30">
-        <f>IF($F120="","",IF($F120&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B120),"PR ★",""))</f>
+        <f>IF($F120="","",IF($F120&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B120),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4932,7 +4941,7 @@
         <v/>
       </c>
       <c r="G121" s="30">
-        <f>IF($F121="","",IF($F121&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B121),"PR ★",""))</f>
+        <f>IF($F121="","",IF($F121&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B121),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4944,7 +4953,7 @@
         <v/>
       </c>
       <c r="G122" s="30">
-        <f>IF($F122="","",IF($F122&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B122),"PR ★",""))</f>
+        <f>IF($F122="","",IF($F122&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B122),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4956,7 +4965,7 @@
         <v/>
       </c>
       <c r="G123" s="30">
-        <f>IF($F123="","",IF($F123&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B123),"PR ★",""))</f>
+        <f>IF($F123="","",IF($F123&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B123),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4968,7 +4977,7 @@
         <v/>
       </c>
       <c r="G124" s="30">
-        <f>IF($F124="","",IF($F124&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B124),"PR ★",""))</f>
+        <f>IF($F124="","",IF($F124&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B124),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4980,7 +4989,7 @@
         <v/>
       </c>
       <c r="G125" s="30">
-        <f>IF($F125="","",IF($F125&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B125),"PR ★",""))</f>
+        <f>IF($F125="","",IF($F125&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B125),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -4992,7 +5001,7 @@
         <v/>
       </c>
       <c r="G126" s="30">
-        <f>IF($F126="","",IF($F126&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B126),"PR ★",""))</f>
+        <f>IF($F126="","",IF($F126&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B126),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5004,7 +5013,7 @@
         <v/>
       </c>
       <c r="G127" s="30">
-        <f>IF($F127="","",IF($F127&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B127),"PR ★",""))</f>
+        <f>IF($F127="","",IF($F127&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B127),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5016,7 +5025,7 @@
         <v/>
       </c>
       <c r="G128" s="30">
-        <f>IF($F128="","",IF($F128&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B128),"PR ★",""))</f>
+        <f>IF($F128="","",IF($F128&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B128),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5028,7 +5037,7 @@
         <v/>
       </c>
       <c r="G129" s="30">
-        <f>IF($F129="","",IF($F129&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B129),"PR ★",""))</f>
+        <f>IF($F129="","",IF($F129&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B129),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5040,7 +5049,7 @@
         <v/>
       </c>
       <c r="G130" s="30">
-        <f>IF($F130="","",IF($F130&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B130),"PR ★",""))</f>
+        <f>IF($F130="","",IF($F130&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B130),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5052,7 +5061,7 @@
         <v/>
       </c>
       <c r="G131" s="30">
-        <f>IF($F131="","",IF($F131&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B131),"PR ★",""))</f>
+        <f>IF($F131="","",IF($F131&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B131),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5064,7 +5073,7 @@
         <v/>
       </c>
       <c r="G132" s="30">
-        <f>IF($F132="","",IF($F132&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B132),"PR ★",""))</f>
+        <f>IF($F132="","",IF($F132&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B132),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5076,7 +5085,7 @@
         <v/>
       </c>
       <c r="G133" s="30">
-        <f>IF($F133="","",IF($F133&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B133),"PR ★",""))</f>
+        <f>IF($F133="","",IF($F133&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B133),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5088,7 +5097,7 @@
         <v/>
       </c>
       <c r="G134" s="30">
-        <f>IF($F134="","",IF($F134&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B134),"PR ★",""))</f>
+        <f>IF($F134="","",IF($F134&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B134),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5100,7 +5109,7 @@
         <v/>
       </c>
       <c r="G135" s="30">
-        <f>IF($F135="","",IF($F135&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B135),"PR ★",""))</f>
+        <f>IF($F135="","",IF($F135&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B135),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5112,7 +5121,7 @@
         <v/>
       </c>
       <c r="G136" s="30">
-        <f>IF($F136="","",IF($F136&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B136),"PR ★",""))</f>
+        <f>IF($F136="","",IF($F136&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B136),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5124,7 +5133,7 @@
         <v/>
       </c>
       <c r="G137" s="30">
-        <f>IF($F137="","",IF($F137&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B137),"PR ★",""))</f>
+        <f>IF($F137="","",IF($F137&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B137),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5136,7 +5145,7 @@
         <v/>
       </c>
       <c r="G138" s="30">
-        <f>IF($F138="","",IF($F138&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B138),"PR ★",""))</f>
+        <f>IF($F138="","",IF($F138&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B138),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5148,7 +5157,7 @@
         <v/>
       </c>
       <c r="G139" s="30">
-        <f>IF($F139="","",IF($F139&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B139),"PR ★",""))</f>
+        <f>IF($F139="","",IF($F139&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B139),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5160,7 +5169,7 @@
         <v/>
       </c>
       <c r="G140" s="30">
-        <f>IF($F140="","",IF($F140&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B140),"PR ★",""))</f>
+        <f>IF($F140="","",IF($F140&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B140),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5172,7 +5181,7 @@
         <v/>
       </c>
       <c r="G141" s="30">
-        <f>IF($F141="","",IF($F141&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B141),"PR ★",""))</f>
+        <f>IF($F141="","",IF($F141&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B141),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5184,7 +5193,7 @@
         <v/>
       </c>
       <c r="G142" s="30">
-        <f>IF($F142="","",IF($F142&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B142),"PR ★",""))</f>
+        <f>IF($F142="","",IF($F142&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B142),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5196,7 +5205,7 @@
         <v/>
       </c>
       <c r="G143" s="30">
-        <f>IF($F143="","",IF($F143&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B143),"PR ★",""))</f>
+        <f>IF($F143="","",IF($F143&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B143),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5208,7 +5217,7 @@
         <v/>
       </c>
       <c r="G144" s="30">
-        <f>IF($F144="","",IF($F144&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B144),"PR ★",""))</f>
+        <f>IF($F144="","",IF($F144&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B144),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5220,7 +5229,7 @@
         <v/>
       </c>
       <c r="G145" s="30">
-        <f>IF($F145="","",IF($F145&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B145),"PR ★",""))</f>
+        <f>IF($F145="","",IF($F145&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B145),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5232,7 +5241,7 @@
         <v/>
       </c>
       <c r="G146" s="30">
-        <f>IF($F146="","",IF($F146&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B146),"PR ★",""))</f>
+        <f>IF($F146="","",IF($F146&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B146),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5244,7 +5253,7 @@
         <v/>
       </c>
       <c r="G147" s="30">
-        <f>IF($F147="","",IF($F147&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B147),"PR ★",""))</f>
+        <f>IF($F147="","",IF($F147&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B147),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5256,7 +5265,7 @@
         <v/>
       </c>
       <c r="G148" s="30">
-        <f>IF($F148="","",IF($F148&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B148),"PR ★",""))</f>
+        <f>IF($F148="","",IF($F148&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B148),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5268,7 +5277,7 @@
         <v/>
       </c>
       <c r="G149" s="30">
-        <f>IF($F149="","",IF($F149&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B149),"PR ★",""))</f>
+        <f>IF($F149="","",IF($F149&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B149),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5280,7 +5289,7 @@
         <v/>
       </c>
       <c r="G150" s="30">
-        <f>IF($F150="","",IF($F150&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B150),"PR ★",""))</f>
+        <f>IF($F150="","",IF($F150&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B150),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5292,7 +5301,7 @@
         <v/>
       </c>
       <c r="G151" s="30">
-        <f>IF($F151="","",IF($F151&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B151),"PR ★",""))</f>
+        <f>IF($F151="","",IF($F151&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B151),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5304,7 +5313,7 @@
         <v/>
       </c>
       <c r="G152" s="30">
-        <f>IF($F152="","",IF($F152&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B152),"PR ★",""))</f>
+        <f>IF($F152="","",IF($F152&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B152),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5316,7 +5325,7 @@
         <v/>
       </c>
       <c r="G153" s="30">
-        <f>IF($F153="","",IF($F153&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B153),"PR ★",""))</f>
+        <f>IF($F153="","",IF($F153&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B153),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5328,7 +5337,7 @@
         <v/>
       </c>
       <c r="G154" s="30">
-        <f>IF($F154="","",IF($F154&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B154),"PR ★",""))</f>
+        <f>IF($F154="","",IF($F154&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B154),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5340,7 +5349,7 @@
         <v/>
       </c>
       <c r="G155" s="30">
-        <f>IF($F155="","",IF($F155&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B155),"PR ★",""))</f>
+        <f>IF($F155="","",IF($F155&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B155),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5352,7 +5361,7 @@
         <v/>
       </c>
       <c r="G156" s="30">
-        <f>IF($F156="","",IF($F156&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B156),"PR ★",""))</f>
+        <f>IF($F156="","",IF($F156&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B156),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5364,7 +5373,7 @@
         <v/>
       </c>
       <c r="G157" s="30">
-        <f>IF($F157="","",IF($F157&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B157),"PR ★",""))</f>
+        <f>IF($F157="","",IF($F157&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B157),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5376,7 +5385,7 @@
         <v/>
       </c>
       <c r="G158" s="30">
-        <f>IF($F158="","",IF($F158&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B158),"PR ★",""))</f>
+        <f>IF($F158="","",IF($F158&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B158),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5388,7 +5397,7 @@
         <v/>
       </c>
       <c r="G159" s="30">
-        <f>IF($F159="","",IF($F159&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B159),"PR ★",""))</f>
+        <f>IF($F159="","",IF($F159&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B159),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5400,7 +5409,7 @@
         <v/>
       </c>
       <c r="G160" s="30">
-        <f>IF($F160="","",IF($F160&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B160),"PR ★",""))</f>
+        <f>IF($F160="","",IF($F160&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B160),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5412,7 +5421,7 @@
         <v/>
       </c>
       <c r="G161" s="30">
-        <f>IF($F161="","",IF($F161&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B161),"PR ★",""))</f>
+        <f>IF($F161="","",IF($F161&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B161),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5424,7 +5433,7 @@
         <v/>
       </c>
       <c r="G162" s="30">
-        <f>IF($F162="","",IF($F162&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B162),"PR ★",""))</f>
+        <f>IF($F162="","",IF($F162&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B162),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5436,7 +5445,7 @@
         <v/>
       </c>
       <c r="G163" s="30">
-        <f>IF($F163="","",IF($F163&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B163),"PR ★",""))</f>
+        <f>IF($F163="","",IF($F163&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B163),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5448,7 +5457,7 @@
         <v/>
       </c>
       <c r="G164" s="30">
-        <f>IF($F164="","",IF($F164&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B164),"PR ★",""))</f>
+        <f>IF($F164="","",IF($F164&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B164),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5460,7 +5469,7 @@
         <v/>
       </c>
       <c r="G165" s="30">
-        <f>IF($F165="","",IF($F165&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B165),"PR ★",""))</f>
+        <f>IF($F165="","",IF($F165&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B165),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5472,7 +5481,7 @@
         <v/>
       </c>
       <c r="G166" s="30">
-        <f>IF($F166="","",IF($F166&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B166),"PR ★",""))</f>
+        <f>IF($F166="","",IF($F166&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B166),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5484,7 +5493,7 @@
         <v/>
       </c>
       <c r="G167" s="30">
-        <f>IF($F167="","",IF($F167&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B167),"PR ★",""))</f>
+        <f>IF($F167="","",IF($F167&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B167),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5496,7 +5505,7 @@
         <v/>
       </c>
       <c r="G168" s="30">
-        <f>IF($F168="","",IF($F168&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B168),"PR ★",""))</f>
+        <f>IF($F168="","",IF($F168&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B168),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5508,7 +5517,7 @@
         <v/>
       </c>
       <c r="G169" s="30">
-        <f>IF($F169="","",IF($F169&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B169),"PR ★",""))</f>
+        <f>IF($F169="","",IF($F169&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B169),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5520,7 +5529,7 @@
         <v/>
       </c>
       <c r="G170" s="30">
-        <f>IF($F170="","",IF($F170&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B170),"PR ★",""))</f>
+        <f>IF($F170="","",IF($F170&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B170),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5532,7 +5541,7 @@
         <v/>
       </c>
       <c r="G171" s="30">
-        <f>IF($F171="","",IF($F171&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B171),"PR ★",""))</f>
+        <f>IF($F171="","",IF($F171&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B171),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5544,7 +5553,7 @@
         <v/>
       </c>
       <c r="G172" s="30">
-        <f>IF($F172="","",IF($F172&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B172),"PR ★",""))</f>
+        <f>IF($F172="","",IF($F172&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B172),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5556,7 +5565,7 @@
         <v/>
       </c>
       <c r="G173" s="30">
-        <f>IF($F173="","",IF($F173&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B173),"PR ★",""))</f>
+        <f>IF($F173="","",IF($F173&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B173),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5568,7 +5577,7 @@
         <v/>
       </c>
       <c r="G174" s="30">
-        <f>IF($F174="","",IF($F174&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B174),"PR ★",""))</f>
+        <f>IF($F174="","",IF($F174&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B174),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5580,7 +5589,7 @@
         <v/>
       </c>
       <c r="G175" s="30">
-        <f>IF($F175="","",IF($F175&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B175),"PR ★",""))</f>
+        <f>IF($F175="","",IF($F175&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B175),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5592,7 +5601,7 @@
         <v/>
       </c>
       <c r="G176" s="30">
-        <f>IF($F176="","",IF($F176&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B176),"PR ★",""))</f>
+        <f>IF($F176="","",IF($F176&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B176),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5604,7 +5613,7 @@
         <v/>
       </c>
       <c r="G177" s="30">
-        <f>IF($F177="","",IF($F177&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B177),"PR ★",""))</f>
+        <f>IF($F177="","",IF($F177&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B177),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5616,7 +5625,7 @@
         <v/>
       </c>
       <c r="G178" s="30">
-        <f>IF($F178="","",IF($F178&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B178),"PR ★",""))</f>
+        <f>IF($F178="","",IF($F178&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B178),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5628,7 +5637,7 @@
         <v/>
       </c>
       <c r="G179" s="30">
-        <f>IF($F179="","",IF($F179&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B179),"PR ★",""))</f>
+        <f>IF($F179="","",IF($F179&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B179),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5640,7 +5649,7 @@
         <v/>
       </c>
       <c r="G180" s="30">
-        <f>IF($F180="","",IF($F180&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B180),"PR ★",""))</f>
+        <f>IF($F180="","",IF($F180&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B180),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5652,7 +5661,7 @@
         <v/>
       </c>
       <c r="G181" s="30">
-        <f>IF($F181="","",IF($F181&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B181),"PR ★",""))</f>
+        <f>IF($F181="","",IF($F181&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B181),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5664,7 +5673,7 @@
         <v/>
       </c>
       <c r="G182" s="30">
-        <f>IF($F182="","",IF($F182&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B182),"PR ★",""))</f>
+        <f>IF($F182="","",IF($F182&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B182),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5676,7 +5685,7 @@
         <v/>
       </c>
       <c r="G183" s="30">
-        <f>IF($F183="","",IF($F183&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B183),"PR ★",""))</f>
+        <f>IF($F183="","",IF($F183&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B183),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5688,7 +5697,7 @@
         <v/>
       </c>
       <c r="G184" s="30">
-        <f>IF($F184="","",IF($F184&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B184),"PR ★",""))</f>
+        <f>IF($F184="","",IF($F184&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B184),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5700,7 +5709,7 @@
         <v/>
       </c>
       <c r="G185" s="30">
-        <f>IF($F185="","",IF($F185&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B185),"PR ★",""))</f>
+        <f>IF($F185="","",IF($F185&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B185),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5712,7 +5721,7 @@
         <v/>
       </c>
       <c r="G186" s="30">
-        <f>IF($F186="","",IF($F186&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B186),"PR ★",""))</f>
+        <f>IF($F186="","",IF($F186&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B186),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5724,7 +5733,7 @@
         <v/>
       </c>
       <c r="G187" s="30">
-        <f>IF($F187="","",IF($F187&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B187),"PR ★",""))</f>
+        <f>IF($F187="","",IF($F187&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B187),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5736,7 +5745,7 @@
         <v/>
       </c>
       <c r="G188" s="30">
-        <f>IF($F188="","",IF($F188&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B188),"PR ★",""))</f>
+        <f>IF($F188="","",IF($F188&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B188),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5748,7 +5757,7 @@
         <v/>
       </c>
       <c r="G189" s="30">
-        <f>IF($F189="","",IF($F189&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B189),"PR ★",""))</f>
+        <f>IF($F189="","",IF($F189&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B189),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5760,7 +5769,7 @@
         <v/>
       </c>
       <c r="G190" s="30">
-        <f>IF($F190="","",IF($F190&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B190),"PR ★",""))</f>
+        <f>IF($F190="","",IF($F190&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B190),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5772,7 +5781,7 @@
         <v/>
       </c>
       <c r="G191" s="30">
-        <f>IF($F191="","",IF($F191&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B191),"PR ★",""))</f>
+        <f>IF($F191="","",IF($F191&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B191),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5784,7 +5793,7 @@
         <v/>
       </c>
       <c r="G192" s="30">
-        <f>IF($F192="","",IF($F192&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B192),"PR ★",""))</f>
+        <f>IF($F192="","",IF($F192&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B192),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5796,7 +5805,7 @@
         <v/>
       </c>
       <c r="G193" s="30">
-        <f>IF($F193="","",IF($F193&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B193),"PR ★",""))</f>
+        <f>IF($F193="","",IF($F193&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B193),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5808,7 +5817,7 @@
         <v/>
       </c>
       <c r="G194" s="30">
-        <f>IF($F194="","",IF($F194&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B194),"PR ★",""))</f>
+        <f>IF($F194="","",IF($F194&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B194),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5820,7 +5829,7 @@
         <v/>
       </c>
       <c r="G195" s="30">
-        <f>IF($F195="","",IF($F195&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B195),"PR ★",""))</f>
+        <f>IF($F195="","",IF($F195&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B195),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5832,7 +5841,7 @@
         <v/>
       </c>
       <c r="G196" s="30">
-        <f>IF($F196="","",IF($F196&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B196),"PR ★",""))</f>
+        <f>IF($F196="","",IF($F196&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B196),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5844,7 +5853,7 @@
         <v/>
       </c>
       <c r="G197" s="30">
-        <f>IF($F197="","",IF($F197&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B197),"PR ★",""))</f>
+        <f>IF($F197="","",IF($F197&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B197),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5856,7 +5865,7 @@
         <v/>
       </c>
       <c r="G198" s="30">
-        <f>IF($F198="","",IF($F198&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B198),"PR ★",""))</f>
+        <f>IF($F198="","",IF($F198&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B198),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5868,7 +5877,7 @@
         <v/>
       </c>
       <c r="G199" s="30">
-        <f>IF($F199="","",IF($F199&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B199),"PR ★",""))</f>
+        <f>IF($F199="","",IF($F199&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B199),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5880,7 +5889,7 @@
         <v/>
       </c>
       <c r="G200" s="30">
-        <f>IF($F200="","",IF($F200&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B200),"PR ★",""))</f>
+        <f>IF($F200="","",IF($F200&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B200),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5892,7 +5901,7 @@
         <v/>
       </c>
       <c r="G201" s="30">
-        <f>IF($F201="","",IF($F201&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B201),"PR ★",""))</f>
+        <f>IF($F201="","",IF($F201&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B201),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5904,7 +5913,7 @@
         <v/>
       </c>
       <c r="G202" s="30">
-        <f>IF($F202="","",IF($F202&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B202),"PR ★",""))</f>
+        <f>IF($F202="","",IF($F202&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B202),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5916,7 +5925,7 @@
         <v/>
       </c>
       <c r="G203" s="30">
-        <f>IF($F203="","",IF($F203&gt;=MAXIFS($F$4:$F$203,$B$4:$B$203,$B203),"PR ★",""))</f>
+        <f>IF($F203="","",IF($F203&gt;=_xlfn.MAXIFS($F$4:$F$203,$B$4:$B$203,$B203),"PR ★",""))</f>
         <v/>
       </c>
     </row>
@@ -5929,7 +5938,8 @@
       <formula1>=$I$4:$I$23</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -5939,7 +5949,7 @@
   <sheetPr>
     <tabColor rgb="0016A34A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -6077,6 +6087,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>